<commit_message>
fix(AASPGOV01): corrige GEST xlsx e adiciona RDP v3.0
- GEST-AASPGOV01: regenerado com JSZip (paths forward-slash) — arquivo anterior
  estava corrompido por Compress-Archive do PowerShell (backslash paths)
- RDP-AASPGOV01-001 v3.0: criado a partir do v2.0 com atualizacoes:
  * Todos os codigos AASP-GOV- corrigidos para AASPGOV01- (36 ocorrencias)
  * Auditor: Jonathan Barbosa -> Jonathan Alves
  * Versao 3.0 — 14/06/2026
  * Gerente de Projeto: Abraao Oliveira (separado de Tech Lead = Cezar Hiraki)
  * Equipe completa: Caroline Sousa, Lucas Batista, Jonathan Alves adicionados
  * Sprints S0-S3 no lugar de Fases para alinhamento retroativo
  * CT-06 a CT-12 adicionados (total 12 CTs: 8 happy, 4 sad)
  * GQA items 11-16 adicionados (total 16 itens verificados)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Automacao-Governanca/GEST-AASPGOV01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Automacao-Governanca/GEST-AASPGOV01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -1,20 +1,28 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties">
-  <Application>Microsoft Excel Compatible / Openpyxl 3.1.5</Application>
-  <AppVersion>3.1</AppVersion>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Visão Geral" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cronograma" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Backlog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Equipe" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Acompanhamento" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Riscos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Medição" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="GQA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="V&amp;V — Testes" sheetId="9" state="visible" r:id="rId9"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
-  <dc:creator>openpyxl</dc:creator>
-  <dcterms:created xsi:type="dcterms:W3CDTF">2026-06-05T23:07:58Z</dcterms:created>
-  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-06-05T23:22:11Z</dcterms:modified>
-</cp:coreProperties>
-</file>
-
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
   <fonts count="18">
@@ -449,7 +457,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -732,30 +740,7 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Visão Geral" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cronograma" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Backlog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Equipe" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Acompanhamento" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Riscos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Medição" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="GQA" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="V&amp;V — Testes" sheetId="9" state="visible" r:id="rId9"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1215,7 +1200,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1596,7 +1581,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2401,7 +2386,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2726,7 +2711,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3261,7 +3246,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3627,7 +3612,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3931,7 +3916,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4546,7 +4531,7 @@
 </worksheet>
 </file>
 
-<file path=xl\worksheets\sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs(GEST): atualizar planilha de gestão com nova composição de equipe
Abas atualizadas:
- Visão Geral: Referência GQA → Caroline Sousa (GQA Independente)
- Equipe: Cezar ganha DevOps/Arquiteto; Henry substituiu Raony; Jonatan como QA;
  Felipe substituiu Lucas Batista; Caroline Sousa como GQA Independente no lugar de Jonathan Alves
- GQA: auditor atualizado de Jonathan Alves para Caroline Sousa (GQA Independente);
  item 8 onboarding: Caroline → Jonatan

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Automacao-Governanca/GEST-AASPGOV01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Automacao-Governanca/GEST-AASPGOV01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -746,6 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -769,6 +770,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -844,10 +846,11 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>GQA-AASPGOV01-001 (Auditor: Jonathan Alves — independente)</t>
-        </is>
-      </c>
-    </row>
+          <t>GQA-AASPGOV01-001 (GQA Independente: Caroline Sousa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
@@ -965,6 +968,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -1190,11 +1194,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1206,6 +1210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1587,6 +1592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2378,9 +2384,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A4:H4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2392,6 +2398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2416,6 +2423,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2480,7 +2488,7 @@
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t>Cezar Hiraki · Tech Lead / Dev</t>
+          <t>Cezar Hiraki · Tech Lead / DevOps / Arquiteto</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
@@ -2507,7 +2515,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Raony Chagas · Dev (.NET)</t>
+          <t>Henry · Dev (.NET)</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -2517,7 +2525,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>S0–S2</t>
+          <t>S0–S3</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -2527,7 +2535,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Sprints S0–S2; pipeline de migração</t>
+          <t>Sprints S0–S3; pipeline de migração</t>
         </is>
       </c>
     </row>
@@ -2561,17 +2569,17 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Caroline Sousa · Dev (.NET)</t>
+          <t>Jonatan · QA</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Desenvolvimento logging, error handling e retry</t>
+          <t>Homologação, testes E2E e validação de aceite</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>S1–S3</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -2588,17 +2596,17 @@
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Lucas Batista · Dev (.NET)</t>
+          <t>Felipe · Dev (.NET)</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>V&amp;V, testes de integração e documentação técnica</t>
+          <t>Desenvolvimento e suporte ao pipeline de transformação e integração</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>S2–S3</t>
+          <t>S1–S3</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -2608,14 +2616,14 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Suporte VV e redação REL-VV</t>
+          <t>Onboarding 17/04/2026; CAP-AASPGOV01-001</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Jonathan Alves · Auditor GQA</t>
+          <t>Caroline Sousa · GQA Independente</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -2639,6 +2647,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
@@ -2717,6 +2726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2941,7 +2951,7 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -2956,7 +2966,7 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>RF-03, RF-04, RF-06, RF-09 a RF-11 entregues; BUG-01 a BUG-05 resolvidos</t>
+          <t>RF-03, RF-04, RF-06, RF-09 a RF-11 entregues</t>
         </is>
       </c>
     </row>
@@ -2993,14 +3003,14 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
           <t>100%</t>
@@ -3008,7 +3018,7 @@
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>12 CTs aprovados; CA01–CA07 validados; 0 defeitos escapados para produção</t>
+          <t>12 CTs aprovados; CA01–CA07 validados; BUG-01 a BUG-05 identificados e resolvidos; 0 defeitos escapados para produção</t>
         </is>
       </c>
     </row>
@@ -3171,16 +3181,8 @@
           <t>Status</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -3223,24 +3225,16 @@
           <t>N/A</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J17" s="7" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="I17" s="7" t="inlineStr"/>
+      <c r="J17" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A15:J15"/>
+    <mergeCell ref="A4:J4"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A4:J4"/>
     <mergeCell ref="A11:J11"/>
-    <mergeCell ref="A15:J15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3252,6 +3246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3604,9 +3599,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A4:J4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3618,6 +3613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3908,9 +3904,9 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3922,6 +3918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3941,10 +3938,11 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Referência: GQA-AASPGOV01-001 · EST-GPC-001 · TPL-GPC-001 · Auditor: Jonathan Alves — independente da equipe de projeto</t>
-        </is>
-      </c>
-    </row>
+          <t>Referência: GQA-AASPGOV01-001 · EST-GPC-001 · TPL-GPC-001 · GQA Independente: Caroline Sousa — independente da equipe de projeto</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -3953,7 +3951,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Jonathan Alves (Auditor GQA)</t>
+          <t>Caroline Sousa (GQA Independente)</t>
         </is>
       </c>
     </row>
@@ -3965,7 +3963,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Sim — Jonathan Alves não participou da execução do projeto em nenhuma fase</t>
+          <t>Sim — Caroline Sousa (GQA Independente) não participou da execução do projeto como membro do time de desenvolvimento</t>
         </is>
       </c>
     </row>
@@ -3993,6 +3991,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
@@ -4239,7 +4238,7 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Onboarding Allan (17/04) e Caroline (21/05)</t>
+          <t>Onboarding Allan (17/04) e Jonatan (21/05)</t>
         </is>
       </c>
     </row>
@@ -4459,6 +4458,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -4522,10 +4522,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A9:E9"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A28:E28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4537,6 +4537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5407,8 +5408,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A17:J17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(GEST): corrige grafia Jonathan no GEST xlsx (Equipe!A10 e GQA!E18)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/04_registros/AASP_Automacao-Governanca/GEST-AASPGOV01_Planilha-de-Gestao-do-Projeto.xlsx
+++ b/mps-nivel-c/oficial/04_registros/AASP_Automacao-Governanca/GEST-AASPGOV01_Planilha-de-Gestao-do-Projeto.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Visão Geral" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cronograma" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Backlog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Equipe" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Acompanhamento" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Riscos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Medição" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="GQA" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="V&amp;V — Testes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Visão Geral" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipe" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acompanhamento" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riscos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Medição" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GQA" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="V&amp;V — Testes" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1236,6 +1236,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1619,6 +1620,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2569,7 +2571,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Jonatan · QA</t>
+          <t>Jonathan · QA</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -2755,6 +2757,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3022,6 +3025,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -3133,6 +3137,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -3275,6 +3280,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3639,6 +3645,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4238,7 +4245,7 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>Onboarding Allan (17/04) e Jonatan (21/05)</t>
+          <t>Onboarding Allan (17/04) e Jonathan (21/05)</t>
         </is>
       </c>
     </row>
@@ -5270,6 +5277,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="15" t="inlineStr">
         <is>
@@ -5407,8 +5415,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>